<commit_message>
docs: actualizar guía de importación CSV y template XLSX
Actualizar documentación y template para reflejar los nuevos campos
de importación (items_sin_iva, importe_neto).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/public/templates/facturas_template.xlsx
+++ b/frontend/public/templates/facturas_template.xlsx
@@ -1,14 +1,415 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="facturas" sheetId="1" r:id="rId1"/>
+    <sheet name="facturas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="1">
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+  </fonts>
+  <fills count="2">
+    <fill>
+      <patternFill/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+  </cellStyles>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
+</styleSheet>
+</file>
+
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -106,11 +507,6 @@
           <t>item_precio_unitario</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>item_alicuota_iva_id</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -148,21 +544,9 @@
           <t>100.00</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr">
         <is>
           <t>21.00</t>
@@ -178,21 +562,9 @@
           <t>1</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
       <c r="Q2" t="inlineStr">
         <is>
           <t>Servicio mensual</t>
@@ -206,14 +578,10 @@
       <c r="S2" t="inlineStr">
         <is>
           <t>100</t>
-        </is>
-      </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>5</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: eliminar facturador_cuit del CSV e importar facturador desde modal
- Remover facturador_cuit de columnas requeridas y parser CSV
- Recibir facturador_id desde form data en endpoint de importación
- Agregar dropdown de facturador en ImportModal
- Regenerar template XLSX sin columna facturador_cuit
- Actualizar documentación de importación
- Actualizar tests (csv_parser, facturas, lotes)
</commit_message>
<xml_diff>
--- a/frontend/public/templates/facturas_template.xlsx
+++ b/frontend/public/templates/facturas_template.xlsx
@@ -2,17 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
     <sheet name="facturas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -20,16 +25,30 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -37,12 +56,32 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B4C6E7"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B4C6E7"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B4C6E7"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B4C6E7"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -408,176 +447,346 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="25" customWidth="1" min="16" max="16"/>
+    <col width="17" customWidth="1" min="17" max="17"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>facturador_cuit</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>receptor_cuit</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>tipo_comprobante</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>concepto</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>fecha_emision</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>importe_total</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>importe_neto</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>fecha_desde</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>fecha_hasta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>fecha_vto_pago</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>importe_iva</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>moneda</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>cotizacion</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>cbte_asoc_tipo</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>cbte_asoc_pto_vta</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>cbte_asoc_nro</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>item_descripcion</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>item_cantidad</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>item_precio_unitario</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>20123456789</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>27293188217</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>2026-02-09</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>121.00</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>100.00</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="inlineStr">
         <is>
           <t>21.00</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>PES</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="inlineStr">
         <is>
           <t>Servicio mensual</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>100</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>27293188217</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>121.00</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>100.00</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="n"/>
+      <c r="H3" s="2" t="n"/>
+      <c r="I3" s="2" t="n"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>21.00</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>PES</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Soporte técnico</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>30712345678</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>242.00</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>200.00</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-01</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-15</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>42.00</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>PES</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Ajuste por diferencia</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>200</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: items obligatorios en CSV, validación cruzada de importes y eliminar moneda/cotización
</commit_message>
<xml_diff>
--- a/frontend/public/templates/facturas_template.xlsx
+++ b/frontend/public/templates/facturas_template.xlsx
@@ -2,17 +2,22 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
+  <bookViews>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+  </bookViews>
   <sheets>
-    <sheet name="facturas" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Facturas" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -20,16 +25,32 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -37,12 +58,24 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -408,178 +441,234 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:P4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>facturador_cuit</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>receptor_cuit</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>tipo_comprobante</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>concepto</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>fecha_emision</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>importe_total</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>importe_neto</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>importe_iva</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>item_descripcion</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>item_cantidad</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>item_precio_unitario</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>fecha_desde</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>fecha_hasta</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>fecha_vto_pago</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>importe_iva</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>moneda</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>cotizacion</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>cbte_asoc_tipo</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>cbte_asoc_pto_vta</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>cbte_asoc_nro</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>item_descripcion</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>item_cantidad</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>item_precio_unitario</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>20123456789</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>27293188217</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>2026-02-09</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>121.00</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>100.00</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>21.00</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>PES</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>Servicio mensual</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="S2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="n">
+        <v>20222222223</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>1210</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G2" s="2" t="n">
+        <v>210</v>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Servicios Profesionales</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" s="2" t="n">
+        <v>1000</v>
+      </c>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>20222222223</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>605</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Consultoría adicional</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>500</v>
+      </c>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="n"/>
+      <c r="N3" s="2" t="n"/>
+      <c r="O3" s="2" t="n"/>
+      <c r="P3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>20333333334</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Servicios monotributo</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>5000</v>
+      </c>
+      <c r="K4" s="2" t="n"/>
+      <c r="L4" s="2" t="n"/>
+      <c r="M4" s="2" t="n"/>
+      <c r="N4" s="2" t="n"/>
+      <c r="O4" s="2" t="n"/>
+      <c r="P4" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix(email): fix override body, dispatch logic, date timezone, and resend UI
- Remove config saludo/despedida from CSV override email body (literal CSV content only)
- Decouple use_factura_overrides from emails_cc presence in dispatch logic
- Fix date-only ISO string timezone parsing in formatDate/formatDateShort
- Show email send button for all authorized facturas regardless of receptor.email
- Open email modal for manual recipient entry when receptor.email is NULL
- Pre-load emails_cc in resend modal destinatarios
- Pre-fill modal with CSV override fields when available
- Update facturas template: remove moneda/cotizacion, add email columns
</commit_message>
<xml_diff>
--- a/frontend/public/templates/facturas_template.xlsx
+++ b/frontend/public/templates/facturas_template.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R4"/>
+  <dimension ref="A1:T4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -460,14 +460,16 @@
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
     <col width="17" customWidth="1" min="15" max="15"/>
-    <col width="25" customWidth="1" min="16" max="16"/>
-    <col width="17" customWidth="1" min="17" max="17"/>
-    <col width="24" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -523,42 +525,52 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>moneda</t>
+          <t>cbte_asoc_tipo</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>cotizacion</t>
+          <t>cbte_asoc_pto_vta</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>cbte_asoc_tipo</t>
+          <t>cbte_asoc_nro</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>cbte_asoc_pto_vta</t>
+          <t>item_descripcion</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>cbte_asoc_nro</t>
+          <t>item_cantidad</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>item_descripcion</t>
+          <t>item_precio_unitario</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>item_cantidad</t>
+          <t>emails_cc</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>item_precio_unitario</t>
+          <t>email_asunto</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>email_mensaje</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>email_firma</t>
         </is>
       </c>
     </row>
@@ -601,30 +613,20 @@
           <t>21.00</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
-          <t>PES</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Servicio mensual</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
-      <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>Servicio mensual</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>100</t>
         </is>
@@ -669,30 +671,20 @@
           <t>21.00</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>PES</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="K3" s="2" t="n"/>
+      <c r="L3" s="2" t="n"/>
       <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
-      <c r="O3" s="2" t="n"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Soporte técnico</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
       <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>Soporte técnico</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="R3" s="2" t="inlineStr">
         <is>
           <t>50</t>
         </is>
@@ -751,7 +743,7 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>PES</t>
+          <t>1</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
@@ -761,30 +753,20 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
+          <t>100</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>Ajuste por diferencia</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
           <t>1</t>
         </is>
       </c>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
       <c r="P4" s="2" t="inlineStr">
-        <is>
-          <t>Ajuste por diferencia</t>
-        </is>
-      </c>
-      <c r="Q4" s="2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>200</t>
         </is>

</xml_diff>